<commit_message>
feat(EM): memory module rework
</commit_message>
<xml_diff>
--- a/Emmersive/package/LangMod/EN/emmersive_localizations.xlsx
+++ b/Emmersive/package/LangMod/EN/emmersive_localizations.xlsx
@@ -2569,12 +2569,12 @@
       </c>
       <c r="C124" s="4" t="inlineStr">
         <is>
-          <t>要約が完了し、長期記憶を{0}件追加しました</t>
+          <t>要約が完了し、長期記憶を{0}件追加・更新しました</t>
         </is>
       </c>
       <c r="D124" s="4" t="inlineStr">
         <is>
-          <t>Summary done: {0} new fact(s) added</t>
+          <t>Summary done: {0} fact(s) added or updated</t>
         </is>
       </c>
     </row>

</xml_diff>